<commit_message>
Partially filled university details from PDF
</commit_message>
<xml_diff>
--- a/university_details_template.xlsx
+++ b/university_details_template.xlsx
@@ -492,7 +492,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Dares Salaam</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -502,7 +502,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -783,7 +783,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non- University</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non- University</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -934,12 +934,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Dodoma</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non-</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -960,12 +960,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Dodoma</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non-</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -986,12 +986,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Dodoma</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non-</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1012,12 +1012,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Dodoma</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non-</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non- University</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non- University</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Shinyanga</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Dodoma</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non- University</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1584,12 +1584,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Pemba</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non-</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Mwanza</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Kilimanjaro</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non- University</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Iringa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2104,12 +2104,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Mbeya</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non- University</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Mbeya</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Arusha</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Arusha</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Dodoma</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Dar es Salaam</t>
+          <t>Iringa</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Government</t>
+          <t>Private</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Non- University</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">

</xml_diff>